<commit_message>
valuation of tinghare and estimate of bajrayogini provided
</commit_message>
<xml_diff>
--- a/बजेट माग estimate/नगर बजेट estimate/bhotange chihaanpaati/bhotange chihaanpaati.xlsx
+++ b/बजेट माग estimate/नगर बजेट estimate/bhotange chihaanpaati/bhotange chihaanpaati.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74D6C1DE-76B2-4520-BF16-96575F97E8D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB733EAF-A4F9-477B-BE11-ECBA2198FB0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,6 +32,8 @@
     <definedName name="description_781">#REF!</definedName>
     <definedName name="description_783">[1]Abstract!$B$301</definedName>
     <definedName name="description_784">[3]Abstract!$B$300</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">estimate!$A$1:$K$158</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">estimate!$1:$8</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -342,10 +344,10 @@
     </r>
   </si>
   <si>
-    <t>Date:2082/09/13</t>
-  </si>
-  <si>
     <t>h/3*(A1+A2+sqrt(A1*A2))</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Date:                  </t>
   </si>
 </sst>
 </file>
@@ -527,7 +529,7 @@
     <xf numFmtId="9" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -639,6 +641,22 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -661,22 +679,9 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -1218,113 +1223,113 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="47" t="s">
+      <c r="A1" s="53" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="47"/>
-      <c r="C1" s="47"/>
-      <c r="D1" s="47"/>
-      <c r="E1" s="47"/>
-      <c r="F1" s="47"/>
-      <c r="G1" s="47"/>
-      <c r="H1" s="47"/>
-      <c r="I1" s="47"/>
-      <c r="J1" s="47"/>
-      <c r="K1" s="47"/>
+      <c r="B1" s="53"/>
+      <c r="C1" s="53"/>
+      <c r="D1" s="53"/>
+      <c r="E1" s="53"/>
+      <c r="F1" s="53"/>
+      <c r="G1" s="53"/>
+      <c r="H1" s="53"/>
+      <c r="I1" s="53"/>
+      <c r="J1" s="53"/>
+      <c r="K1" s="53"/>
     </row>
     <row r="2" spans="1:11" ht="22.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="48" t="s">
+      <c r="A2" s="54" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="48"/>
-      <c r="C2" s="48"/>
-      <c r="D2" s="48"/>
-      <c r="E2" s="48"/>
-      <c r="F2" s="48"/>
-      <c r="G2" s="48"/>
-      <c r="H2" s="48"/>
-      <c r="I2" s="48"/>
-      <c r="J2" s="48"/>
-      <c r="K2" s="48"/>
+      <c r="B2" s="54"/>
+      <c r="C2" s="54"/>
+      <c r="D2" s="54"/>
+      <c r="E2" s="54"/>
+      <c r="F2" s="54"/>
+      <c r="G2" s="54"/>
+      <c r="H2" s="54"/>
+      <c r="I2" s="54"/>
+      <c r="J2" s="54"/>
+      <c r="K2" s="54"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="49" t="s">
+      <c r="A3" s="55" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="49"/>
-      <c r="C3" s="49"/>
-      <c r="D3" s="49"/>
-      <c r="E3" s="49"/>
-      <c r="F3" s="49"/>
-      <c r="G3" s="49"/>
-      <c r="H3" s="49"/>
-      <c r="I3" s="49"/>
-      <c r="J3" s="49"/>
-      <c r="K3" s="49"/>
+      <c r="B3" s="55"/>
+      <c r="C3" s="55"/>
+      <c r="D3" s="55"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="55"/>
+      <c r="G3" s="55"/>
+      <c r="H3" s="55"/>
+      <c r="I3" s="55"/>
+      <c r="J3" s="55"/>
+      <c r="K3" s="55"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="49" t="s">
+      <c r="A4" s="55" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="49"/>
-      <c r="C4" s="49"/>
-      <c r="D4" s="49"/>
-      <c r="E4" s="49"/>
-      <c r="F4" s="49"/>
-      <c r="G4" s="49"/>
-      <c r="H4" s="49"/>
-      <c r="I4" s="49"/>
-      <c r="J4" s="49"/>
-      <c r="K4" s="49"/>
+      <c r="B4" s="55"/>
+      <c r="C4" s="55"/>
+      <c r="D4" s="55"/>
+      <c r="E4" s="55"/>
+      <c r="F4" s="55"/>
+      <c r="G4" s="55"/>
+      <c r="H4" s="55"/>
+      <c r="I4" s="55"/>
+      <c r="J4" s="55"/>
+      <c r="K4" s="55"/>
     </row>
     <row r="5" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A5" s="50" t="s">
+      <c r="A5" s="56" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="50"/>
-      <c r="C5" s="50"/>
-      <c r="D5" s="50"/>
-      <c r="E5" s="50"/>
-      <c r="F5" s="50"/>
-      <c r="G5" s="50"/>
-      <c r="H5" s="50"/>
-      <c r="I5" s="50"/>
-      <c r="J5" s="50"/>
-      <c r="K5" s="50"/>
+      <c r="B5" s="56"/>
+      <c r="C5" s="56"/>
+      <c r="D5" s="56"/>
+      <c r="E5" s="56"/>
+      <c r="F5" s="56"/>
+      <c r="G5" s="56"/>
+      <c r="H5" s="56"/>
+      <c r="I5" s="56"/>
+      <c r="J5" s="56"/>
+      <c r="K5" s="56"/>
     </row>
     <row r="6" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A6" s="51" t="s">
+      <c r="A6" s="57" t="s">
         <v>86</v>
       </c>
-      <c r="B6" s="51"/>
-      <c r="C6" s="51"/>
-      <c r="D6" s="51"/>
-      <c r="E6" s="51"/>
-      <c r="F6" s="51"/>
+      <c r="B6" s="57"/>
+      <c r="C6" s="57"/>
+      <c r="D6" s="57"/>
+      <c r="E6" s="57"/>
+      <c r="F6" s="57"/>
       <c r="G6" s="4"/>
-      <c r="H6" s="52" t="s">
+      <c r="H6" s="58" t="s">
         <v>25</v>
       </c>
-      <c r="I6" s="52"/>
-      <c r="J6" s="52"/>
-      <c r="K6" s="52"/>
+      <c r="I6" s="58"/>
+      <c r="J6" s="58"/>
+      <c r="K6" s="58"/>
     </row>
     <row r="7" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="45" t="s">
+      <c r="A7" s="51" t="s">
         <v>29</v>
       </c>
-      <c r="B7" s="45"/>
-      <c r="C7" s="45"/>
-      <c r="D7" s="45"/>
-      <c r="E7" s="45"/>
-      <c r="F7" s="45"/>
+      <c r="B7" s="51"/>
+      <c r="C7" s="51"/>
+      <c r="D7" s="51"/>
+      <c r="E7" s="51"/>
+      <c r="F7" s="51"/>
       <c r="G7" s="5"/>
-      <c r="H7" s="46" t="s">
-        <v>87</v>
-      </c>
-      <c r="I7" s="46"/>
-      <c r="J7" s="46"/>
-      <c r="K7" s="46"/>
+      <c r="H7" s="52" t="s">
+        <v>88</v>
+      </c>
+      <c r="I7" s="52"/>
+      <c r="J7" s="52"/>
+      <c r="K7" s="52"/>
     </row>
     <row r="8" spans="1:11" s="10" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
@@ -1934,7 +1939,7 @@
       <c r="J34" s="15"/>
       <c r="K34" s="15"/>
       <c r="M34" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.25">
@@ -3305,7 +3310,7 @@
       <c r="H88" s="21" t="s">
         <v>42</v>
       </c>
-      <c r="I88" s="2">
+      <c r="I88" s="59">
         <v>132360</v>
       </c>
       <c r="J88" s="22">
@@ -3520,7 +3525,7 @@
       <c r="B100" s="16" t="s">
         <v>67</v>
       </c>
-      <c r="C100" s="58">
+      <c r="C100" s="45">
         <f>2*2</f>
         <v>4</v>
       </c>
@@ -3545,7 +3550,7 @@
     <row r="101" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A101" s="15"/>
       <c r="B101" s="16"/>
-      <c r="C101" s="58">
+      <c r="C101" s="45">
         <f>2*C117</f>
         <v>4</v>
       </c>
@@ -3573,7 +3578,7 @@
         <f>B119</f>
         <v>-deduction for window</v>
       </c>
-      <c r="C102" s="58">
+      <c r="C102" s="45">
         <f>2*C119</f>
         <v>-4</v>
       </c>
@@ -3601,7 +3606,7 @@
         <f>B120</f>
         <v>-deduction for chain gate</v>
       </c>
-      <c r="C103" s="58">
+      <c r="C103" s="45">
         <f>2*C120</f>
         <v>-2</v>
       </c>
@@ -3850,7 +3855,7 @@
       <c r="E115" s="3">
         <v>0.23</v>
       </c>
-      <c r="F115" s="15">
+      <c r="F115" s="3">
         <v>0.9</v>
       </c>
       <c r="G115" s="3">
@@ -4247,7 +4252,7 @@
         <v>104.43099608071037</v>
       </c>
       <c r="H132" s="21" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="I132" s="2">
         <v>253.8</v>
@@ -4379,7 +4384,7 @@
         <v>3.3441830397713468</v>
       </c>
       <c r="H139" s="21" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="I139" s="2">
         <v>6391.43</v>
@@ -4477,7 +4482,7 @@
         <v>4.9375190490704055</v>
       </c>
       <c r="H144" s="21" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="I144" s="2">
         <v>2485.56</v>
@@ -4627,11 +4632,11 @@
       <c r="B153" s="38" t="s">
         <v>19</v>
       </c>
-      <c r="C153" s="53">
+      <c r="C153" s="46">
         <f>J151</f>
         <v>791637.34255256748</v>
       </c>
-      <c r="D153" s="54"/>
+      <c r="D153" s="47"/>
       <c r="E153" s="39">
         <v>100</v>
       </c>
@@ -4646,21 +4651,21 @@
       <c r="B154" s="38" t="s">
         <v>21</v>
       </c>
-      <c r="C154" s="55">
+      <c r="C154" s="48">
         <v>700000</v>
       </c>
-      <c r="D154" s="56"/>
+      <c r="D154" s="49"/>
       <c r="E154" s="39"/>
     </row>
     <row r="155" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B155" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="C155" s="55">
+      <c r="C155" s="48">
         <f>C154-C157-C158</f>
         <v>665000</v>
       </c>
-      <c r="D155" s="56"/>
+      <c r="D155" s="49"/>
       <c r="E155" s="39">
         <f>C155/C153*100</f>
         <v>84.003111558098539</v>
@@ -4670,11 +4675,11 @@
       <c r="B156" s="38" t="s">
         <v>26</v>
       </c>
-      <c r="C156" s="57">
+      <c r="C156" s="50">
         <f>C153-C155</f>
         <v>126637.34255256748</v>
       </c>
-      <c r="D156" s="57"/>
+      <c r="D156" s="50"/>
       <c r="E156" s="39">
         <f>100-E155</f>
         <v>15.996888441901461</v>
@@ -4684,11 +4689,11 @@
       <c r="B157" s="38" t="s">
         <v>23</v>
       </c>
-      <c r="C157" s="53">
+      <c r="C157" s="46">
         <f>C154*0.03</f>
         <v>21000</v>
       </c>
-      <c r="D157" s="54"/>
+      <c r="D157" s="47"/>
       <c r="E157" s="39">
         <v>3</v>
       </c>
@@ -4697,23 +4702,17 @@
       <c r="B158" s="38" t="s">
         <v>24</v>
       </c>
-      <c r="C158" s="53">
+      <c r="C158" s="46">
         <f>C154*0.02</f>
         <v>14000</v>
       </c>
-      <c r="D158" s="54"/>
+      <c r="D158" s="47"/>
       <c r="E158" s="39">
         <v>2</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="C158:D158"/>
-    <mergeCell ref="C153:D153"/>
-    <mergeCell ref="C154:D154"/>
-    <mergeCell ref="C155:D155"/>
-    <mergeCell ref="C156:D156"/>
-    <mergeCell ref="C157:D157"/>
     <mergeCell ref="A7:F7"/>
     <mergeCell ref="H7:K7"/>
     <mergeCell ref="A1:K1"/>
@@ -4723,8 +4722,17 @@
     <mergeCell ref="A5:K5"/>
     <mergeCell ref="A6:F6"/>
     <mergeCell ref="H6:K6"/>
+    <mergeCell ref="C158:D158"/>
+    <mergeCell ref="C153:D153"/>
+    <mergeCell ref="C154:D154"/>
+    <mergeCell ref="C155:D155"/>
+    <mergeCell ref="C156:D156"/>
+    <mergeCell ref="C157:D157"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup scale="80" orientation="portrait" r:id="rId1"/>
+  <headerFooter>
+    <oddFooter>&amp;LPrepared By:&amp;CChecked By:&amp;RApproved By:</oddFooter>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>